<commit_message>
Email the team when a lead first becomes Hot
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B78hcrBh6is7Ktn7Vptkx9
</commit_message>
<xml_diff>
--- a/digitalhub-messenger-bot/DigitalHub-Chatbot-Sheet-Template.xlsx
+++ b/digitalhub-messenger-bot/DigitalHub-Chatbot-Sheet-Template.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -447,8 +447,9 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,10 +530,15 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Hot Alert Sent</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>